<commit_message>
Separa entrega e depósito no dicionário e evita o RedMine
Cada indicador com as duas vias ganha uma linha por via (entrega no SISMAT,
depósito no Fundo) e uma de total; o RedMine fica só como última opção para
ligar NUP ao processo judicial.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PeYCiidzbNBKwJLDASYnnq
</commit_message>
<xml_diff>
--- a/docs/Dicionario_Painel_Geral_Medicamentos.xlsx
+++ b/docs/Dicionario_Painel_Geral_Medicamentos.xlsx
@@ -492,16 +492,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="42" customWidth="1" min="5" max="5"/>
-    <col width="44" customWidth="1" min="6" max="6"/>
-    <col width="64" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="42" customWidth="1" min="7" max="7"/>
+    <col width="62" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -522,28 +523,35 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>Via</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>Pergunta que responde</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Onde está</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Campos</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Como calcular</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
-        <v>1</v>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
@@ -555,30 +563,37 @@
           <t>Processos que entraram</t>
         </is>
       </c>
-      <c r="D2" s="4" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
         <is>
           <t>Quantos processos chegaram?</t>
         </is>
       </c>
-      <c r="E2" s="4" t="inlineStr">
+      <c r="F2" s="4" t="inlineStr">
         <is>
           <t>Planilha da Triagem (CGAJUD)</t>
         </is>
       </c>
-      <c r="F2" s="4" t="inlineStr">
+      <c r="G2" s="4" t="inlineStr">
         <is>
           <t>NUP · DATA · GRUPO TEMÁTICO · ORIGEM</t>
         </is>
       </c>
-      <c r="G2" s="4" t="inlineStr">
+      <c r="H2" s="4" t="inlineStr">
         <is>
           <t>Contar NUP distintos no período, por mês e por grupo temático.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
-        <v>2</v>
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
@@ -587,33 +602,40 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Viraram depósito</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
+          <t>Cumpridos por depósito</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Depósito (Fundo)</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
         <is>
           <t>Quantos foram cumpridos por depósito e quanto custou?</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="F3" s="4" t="inlineStr">
         <is>
           <t>Fundo · planilha depositos_tratados</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>numero_processo_judicial · data_pagamento · valor_deposito · principio_ativo</t>
-        </is>
-      </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>Contar processos distintos com depósito no período e somar valor_deposito.</t>
+          <t>numero_processo · numero_processo_judicial · data_pagamento · valor_deposito</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>Contar processos distintos (numero_processo_judicial) com data_pagamento no período. Valor = soma de valor_deposito.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n">
-        <v>3</v>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
@@ -622,33 +644,40 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Viraram entrega</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
+          <t>Cumpridos por entrega</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Entrega (SISMAT)</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>Quantos foram cumpridos com entrega do medicamento e quanto custou?</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>SISMAT · djud.gold.tf_saida_material_judicial</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>processo do autor (DS_ENTIDADE) · DT_ENTREGA · QT_ENTREGUE · VL_TOTAL_SAIDA · CO_PROGRAMA_SAUDE · CO_TIPO_MOVIMENTACAO_ESTOQUE</t>
-        </is>
-      </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>Só CO_PROGRAMA_SAUDE = 486 e CO_TIPO_MOVIMENTACAO_ESTOQUE = 6. Contar processos distintos com entrega no período; somar QT_ENTREGUE e VL_TOTAL_SAIDA.</t>
+          <t>DS_ENTIDADE (processo) · DT_ENTREGA · QT_ENTREGUE · VL_TOTAL_SAIDA · CO_PROGRAMA_SAUDE · CO_TIPO_MOVIMENTACAO_ESTOQUE</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>Filtrar CO_PROGRAMA_SAUDE = 486 e CO_TIPO_MOVIMENTACAO_ESTOQUE = 6. Contar processos distintos (DS_ENTIDADE) com DT_ENTREGA no período. Quantidade = soma de QT_ENTREGUE; valor = soma de VL_TOTAL_SAIDA.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n">
-        <v>4</v>
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>4a</t>
+        </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
@@ -657,36 +686,42 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>% cumprido e processos sem cumprimento</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>Quanto do que entrou já foi atendido?</t>
+          <t>% da triagem cumprido por entrega</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Entrega (SISMAT)</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
+          <t>Quanto do que entrou já recebeu o medicamento?</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
           <t>Planilha da Triagem (CGAJUD)
-Fundo · planilha depositos_tratados
-SISMAT · djud.gold.tf_saida_material_judicial
-RedMine · baseRedmine</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>NUP (triagem) · nº do processo judicial (RedMine) · numero_processo_judicial (Fundo) · DS_ENTIDADE (SISMAT)</t>
+SISMAT · djud.gold.tf_saida_material_judicial</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>Ligar o NUP da triagem ao processo judicial pelo RedMine. % cumprido = processos da triagem com depósito ou entrega ÷ processos da triagem. Sem cumprimento = os que não têm nenhum dos dois.</t>
+          <t>Triagem: NUP
+SISMAT: DS_ENTIDADE</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>Ligar NUP da triagem com o processo em DS_ENTIDADE (confirmar se é o NUP 00737). % = NUPs da triagem com entrega ÷ NUPs da triagem.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n">
-        <v>5</v>
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>4b</t>
+        </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
@@ -695,423 +730,758 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Tempo até o cumprimento</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>Quanto tempo leva da entrada ao atendimento?</t>
+          <t>% da triagem cumprido por depósito</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Depósito (Fundo)</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
+          <t>Quanto do que entrou já recebeu depósito?</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
           <t>Planilha da Triagem (CGAJUD)
-Fundo · planilha depositos_tratados
+Fundo · planilha depositos_tratados</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>Triagem: NUP
+Fundo: numero_processo · numero_processo_judicial</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>O Fundo não traz o NUP da triagem (usa o processo de depósito 25000 e o judicial). % = NUPs da triagem com depósito ÷ NUPs da triagem. Para ligar, usar do RedMine apenas o par NUP ↔ nº do processo judicial, se não houver outra ponte.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>4c</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Percurso do processo</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>% cumprido no total e processos sem cumprimento</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Quanto do que entrou ainda não foi atendido?</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>Resultado de 4a e 4b</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>Cumprido = NUP com entrega OU depósito. Sem cumprimento = NUP sem nenhum dos dois. % = cumpridos ÷ NUPs da triagem.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>5a</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Percurso do processo</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Tempo até a entrega</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Entrega (SISMAT)</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>Quanto tempo leva para entregar?</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>Planilha da Triagem (CGAJUD)
 SISMAT · djud.gold.tf_saida_material_judicial</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>DATA (triagem) · data_pagamento · DT_ENTREGA · DT_AUTORIZADO</t>
-        </is>
-      </c>
-      <c r="G6" s="4" t="inlineStr">
-        <is>
-          <t>Entrada → 1º cumprimento = a data mais antiga entre o 1º depósito e a 1ª entrega − DATA da triagem. Autorização → entrega = DT_ENTREGA − DT_AUTORIZADO (descartar datas inválidas como 1-01-01). Mostrar a mediana em dias.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>DATA (triagem) · DT_ENTREGA · DT_AUTORIZADO</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>Entrada → entrega = 1ª DT_ENTREGA do NUP − DATA da triagem. Autorização → entrega = DT_ENTREGA − DT_AUTORIZADO (descartar datas inválidas como 1-01-01). Mostrar a mediana em dias.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>5b</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Percurso do processo</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Tempo até o depósito</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Depósito (Fundo)</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Quanto tempo leva para depositar?</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Planilha da Triagem (CGAJUD)
+Fundo · planilha depositos_tratados</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>DATA (triagem) · data_pagamento</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>Entrada → depósito = 1ª data_pagamento do processo − DATA da triagem (depende da ligação de 4b). Mostrar a mediana em dias.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>6a</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>Por medicamento (CGLJUD)</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>Autores atendidos</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>Quantos autores recebem esse medicamento e por qual via?</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>SISMAT · djud.gold.tf_saida_material_judicial
-Fundo · planilha depositos_tratados</t>
-        </is>
-      </c>
-      <c r="F7" s="4" t="inlineStr">
-        <is>
-          <t>SISMAT: DS_ENTIDADE · DT_ENTREGA · CO_MATERIAL
-Fundo: numero_processo_judicial · data_pagamento · principio_ativo</t>
-        </is>
-      </c>
-      <c r="G7" s="4" t="inlineStr">
-        <is>
-          <t>Processos distintos com entrega + processos distintos com depósito no período, por princípio ativo. Quem aparece nos dois conta uma vez. Ver o passo a passo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="5" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>Autores atendidos por entrega</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Entrega (SISMAT)</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>Quantos autores recebem esse medicamento em espécie?</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>SISMAT · djud.gold.tf_saida_material_judicial</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>DS_ENTIDADE · DT_ENTREGA · CO_MATERIAL</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>Filtrar 486 e tipo 6, DT_ENTREGA no período. Contar processos distintos (DS_ENTIDADE) por princípio ativo (de-para a partir de CO_MATERIAL).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>6b</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>Por medicamento (CGLJUD)</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>Autores atendidos por depósito</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Depósito (Fundo)</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>Quantos autores recebem depósito para esse medicamento?</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>Fundo · planilha depositos_tratados</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>numero_processo_judicial · data_pagamento · principio_ativo</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>data_pagamento no período e principio_ativo diferente de "-" e de "NAO SE APLICA". Contar numero_processo_judicial distintos por princípio ativo (de-para).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>6c</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Por medicamento (CGLJUD)</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>Autores atendidos (total sem duplicar)</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>Quantos autores no total, sem contar duas vezes quem recebeu pelas duas vias?</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>Resultado de 6a e 6b</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>Total = 6a + 6b − autores que aparecem nos dois (mesmo processo nas duas fontes). Pedir ao Vitor a chave que ele já usou.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Por medicamento (CGLJUD)</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
         <is>
           <t>Consumo médio mensal (CMM)</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Entrega (SISMAT)</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
         <is>
           <t>Quanto sai do estoque por mês?</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
+      <c r="F13" s="4" t="inlineStr">
         <is>
           <t>SISMAT · djud.gold.tf_saida_material_judicial</t>
         </is>
       </c>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="G13" s="4" t="inlineStr">
         <is>
           <t>QT_ENTREGUE · DT_SAIDA_MATERIAL · CO_MATERIAL · CO_PROGRAMA_SAUDE · CO_TIPO_MOVIMENTACAO_ESTOQUE</t>
         </is>
       </c>
-      <c r="G8" s="4" t="inlineStr">
-        <is>
-          <t>Soma de QT_ENTREGUE nos últimos 6 meses completos ÷ 6, só 486 e tipo 6. Ver o passo a passo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="5" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>Soma de QT_ENTREGUE nos últimos 6 meses completos ÷ 6, só 486 e tipo 6. Só entrega: depósito não consome estoque. Ver o passo a passo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <t>Por medicamento (CGLJUD)</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="C14" s="6" t="inlineStr">
         <is>
           <t>Cobertura (meses)</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Entrega (SISMAT)</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
         <is>
           <t>Por quanto tempo o estoque atual dura?</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="F14" s="4" t="inlineStr">
         <is>
           <t>SISMAT · djud.gold.tf_estoque_material_judicial
 + indicador 7</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="G14" s="4" t="inlineStr">
         <is>
           <t>saldo do lote · validade · CO_PROGRAMA_SAUDE · CO_MATERIAL</t>
         </is>
       </c>
-      <c r="G9" s="4" t="inlineStr">
+      <c r="H14" s="4" t="inlineStr">
         <is>
           <t>Estoque disponível (486, não vencido) ÷ CMM, por apresentação. Ver o passo a passo.</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="5" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>Por medicamento (CGLJUD)</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>Ata ou contrato vigente e saldo</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
         <is>
           <t>Tenho ata vigente? Quanto ainda posso pedir e por quanto tempo isso dura?</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="F15" s="4" t="inlineStr">
         <is>
           <t>Planilha Gestão de Contratos (SharePoint da CGLJUD) · abas Gerencial e Execução
 SISMAT · dbsismat.bronze.td_material</t>
         </is>
       </c>
-      <c r="F10" s="4" t="inlineStr">
+      <c r="G15" s="4" t="inlineStr">
         <is>
           <t>Gerencial: CATMAT · Nº Contrato · Modalidade · Empresa · Status · Data Assinatura · Vigência · Saldo QTD · Saldo (R$) · Valor Unitário
 td_material: CO_CATMAT · CO_MATERIAL</t>
         </is>
       </c>
-      <c r="G10" s="4" t="inlineStr">
+      <c r="H15" s="4" t="inlineStr">
         <is>
           <t>Contratos com Status = "Ativo", ligados ao material pelo CATMAT. Saldo em quantidade e em R$, data de fim e saldo em meses (saldo ÷ CMM). Ver o passo a passo.</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="5" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>Por medicamento (CGLJUD)</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="C16" s="6" t="inlineStr">
         <is>
           <t>Remanejamentos e recolhimentos</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
         <is>
           <t>Quanto foi remanejado e recolhido, e por quê?</t>
         </is>
       </c>
-      <c r="E11" s="4" t="inlineStr">
+      <c r="F16" s="4" t="inlineStr">
         <is>
           <t>Planilha de Remanejamento/Recolhimento (CGLJUD)</t>
         </is>
       </c>
-      <c r="F11" s="4" t="inlineStr">
+      <c r="G16" s="4" t="inlineStr">
         <is>
           <t>Situação · Medicamento · Motivo · Local de Coleta</t>
         </is>
       </c>
-      <c r="G11" s="4" t="inlineStr">
+      <c r="H16" s="4" t="inlineStr">
         <is>
           <t>Contar registros por Situação (Remanejamento, Recolhimento) e por medicamento no período. Visão resumida; o detalhe fica no painel de remanejamento.</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="5" t="n">
-        <v>11</v>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>Por medicamento (CGLJUD)</t>
         </is>
       </c>
-      <c r="C12" s="6" t="inlineStr">
+      <c r="C17" s="6" t="inlineStr">
         <is>
           <t>Incorporado (RENAME)</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
         <is>
           <t>O medicamento é incorporado?</t>
         </is>
       </c>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="F17" s="4" t="inlineStr">
         <is>
           <t>SISMAT · dbsismat.bronze.td_material</t>
         </is>
       </c>
-      <c r="F12" s="4" t="inlineStr">
+      <c r="G17" s="4" t="inlineStr">
         <is>
           <t>ST_RENAME</t>
         </is>
       </c>
-      <c r="G12" s="4" t="inlineStr">
+      <c r="H17" s="4" t="inlineStr">
         <is>
           <t>Mostrar como coluna e como filtro.</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="7" t="n">
-        <v>12</v>
-      </c>
-      <c r="B13" s="7" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>12a</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
         <is>
           <t>Visão gerencial (Areli)</t>
         </is>
       </c>
-      <c r="C13" s="8" t="inlineStr">
-        <is>
-          <t>Depósito × entrega por mês</t>
-        </is>
-      </c>
-      <c r="D13" s="4" t="inlineStr">
-        <is>
-          <t>Quanto foi gasto por mês em depósitos e em entregas?</t>
-        </is>
-      </c>
-      <c r="E13" s="4" t="inlineStr">
-        <is>
-          <t>Fundo · planilha depositos_tratados
-SISMAT · djud.gold.tf_saida_material_judicial</t>
-        </is>
-      </c>
-      <c r="F13" s="4" t="inlineStr">
-        <is>
-          <t>Fundo: valor_deposito · data_pagamento
-SISMAT: VL_TOTAL_SAIDA · DT_ENTREGA</t>
-        </is>
-      </c>
-      <c r="G13" s="4" t="inlineStr">
-        <is>
-          <t>Somar valor_deposito por mês e VL_TOTAL_SAIDA (486, tipo 6) por mês, lado a lado.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="7" t="n">
-        <v>13</v>
-      </c>
-      <c r="B14" s="7" t="inlineStr">
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>Valor gasto por mês com entrega</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>Entrega (SISMAT)</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>Quanto foi gasto por mês em entregas?</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>SISMAT · djud.gold.tf_saida_material_judicial</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>VL_TOTAL_SAIDA · DT_ENTREGA</t>
+        </is>
+      </c>
+      <c r="H18" s="4" t="inlineStr">
+        <is>
+          <t>Filtrar 486 e tipo 6. Somar VL_TOTAL_SAIDA por mês de DT_ENTREGA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>12b</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
         <is>
           <t>Visão gerencial (Areli)</t>
         </is>
       </c>
-      <c r="C14" s="8" t="inlineStr">
-        <is>
-          <t>Medicamentos mais judicializados por estado</t>
-        </is>
-      </c>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>Valor gasto por mês com depósito</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>Depósito (Fundo)</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>Quanto foi gasto por mês em depósitos?</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>Fundo · planilha depositos_tratados</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>valor_deposito · data_pagamento</t>
+        </is>
+      </c>
+      <c r="H19" s="4" t="inlineStr">
+        <is>
+          <t>Somar valor_deposito por mês de data_pagamento. Mostrar ao lado de 12a.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>13a</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>Visão gerencial (Areli)</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>Medicamentos mais judicializados por estado – depósito</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>Depósito (Fundo)</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
         <is>
           <t>Quais medicamentos mais judicializados em cada UF? E por 100 mil habitantes?</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr">
+      <c r="F20" s="4" t="inlineStr">
         <is>
           <t>Fundo · planilha depositos_tratados
 + população do IBGE</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr">
+      <c r="G20" s="4" t="inlineStr">
         <is>
           <t>uf · principio_ativo · numero_processo_judicial</t>
         </is>
       </c>
-      <c r="G14" s="4" t="inlineStr">
-        <is>
-          <t>Contar processos distintos por UF e medicamento. Por 100 mil hab. = processos da UF ÷ população da UF × 100.000.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="7" t="n">
-        <v>14</v>
-      </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="H20" s="4" t="inlineStr">
+        <is>
+          <t>Contar processos distintos por uf e princípio ativo. Por 100 mil hab. = processos da UF ÷ população da UF × 100.000.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>13b</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
         <is>
           <t>Visão gerencial (Areli)</t>
         </is>
       </c>
-      <c r="C15" s="8" t="inlineStr">
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>Medicamentos mais judicializados por estado – entrega</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>Entrega (SISMAT)</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>Idem, para quem recebe o medicamento</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>Planilha da Triagem (CGAJUD)
+SISMAT · djud.gold.tf_saida_material_judicial</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>Triagem: NUP · UNIDADE FEDERATIVA
+SISMAT: DS_ENTIDADE · CO_MATERIAL</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>O SISMAT não tem UF. Ligar a saída à triagem pelo NUP e usar UNIDADE FEDERATIVA (preenchida só a partir de abril/2026). Contar processos distintos por UF e princípio ativo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>Visão gerencial (Areli)</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="inlineStr">
         <is>
           <t>Tribunais com mais ações</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>Depósito (Fundo)</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
         <is>
           <t>Quais tribunais concentram mais ações e valor?</t>
         </is>
       </c>
-      <c r="E15" s="4" t="inlineStr">
+      <c r="F22" s="4" t="inlineStr">
         <is>
           <t>Fundo · planilha depositos_tratados</t>
         </is>
       </c>
-      <c r="F15" s="4" t="inlineStr">
+      <c r="G22" s="4" t="inlineStr">
         <is>
           <t>numero_processo_judicial · valor_deposito</t>
         </is>
       </c>
-      <c r="G15" s="4" t="inlineStr">
-        <is>
-          <t>Tribunal = dígitos 14 a 16 do número do processo judicial (J + TR). Contar processos e somar valor por tribunal.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="7" t="n">
-        <v>15</v>
-      </c>
-      <c r="B16" s="7" t="inlineStr">
+      <c r="H22" s="4" t="inlineStr">
+        <is>
+          <t>Tribunal = dígitos 14 a 16 do número do processo judicial (J + TR). Contar processos e somar valor_deposito por tribunal. Só depósito: o SISMAT não traz o número judicial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
         <is>
           <t>Visão gerencial (Areli)</t>
         </is>
       </c>
-      <c r="C16" s="8" t="inlineStr">
-        <is>
-          <t>Advogados com mais processos</t>
-        </is>
-      </c>
-      <c r="D16" s="4" t="inlineStr">
-        <is>
-          <t>Quais advogados têm mais processos ativos?</t>
-        </is>
-      </c>
-      <c r="E16" s="4" t="inlineStr">
-        <is>
-          <t>RedMine · baseRedmine</t>
-        </is>
-      </c>
-      <c r="F16" s="4" t="inlineStr">
-        <is>
-          <t>nº da OAB do advogado (a confirmar)</t>
-        </is>
-      </c>
-      <c r="G16" s="4" t="inlineStr">
-        <is>
-          <t>Contar processos por nº da OAB; mostrar os 10 maiores.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="7" t="n">
-        <v>16</v>
-      </c>
-      <c r="B17" s="7" t="inlineStr">
-        <is>
-          <t>Visão gerencial (Areli)</t>
-        </is>
-      </c>
-      <c r="C17" s="8" t="inlineStr">
+      <c r="C23" s="8" t="inlineStr">
         <is>
           <t>Depositar ou comprar</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
         <is>
           <t>Para o mesmo medicamento, sai mais caro depositar ou comprar?</t>
         </is>
       </c>
-      <c r="E17" s="4" t="inlineStr">
+      <c r="F23" s="4" t="inlineStr">
         <is>
           <t>Fundo · planilha depositos_tratados
 Planilha Gestão de Contratos (SharePoint da CGLJUD) · abas Gerencial e Execução</t>
         </is>
       </c>
-      <c r="F17" s="4" t="inlineStr">
-        <is>
-          <t>valor_deposito · Valor Unitário · QT_ENTREGUE</t>
-        </is>
-      </c>
-      <c r="G17" s="4" t="inlineStr">
-        <is>
-          <t>O Fundo não traz quantidade, então comparar por mês de tratamento: depósito ÷ meses cobertos (6; 3 se oncológico) × (quantidade mensal do autor × Valor Unitário do contrato). Estimativa: deixar a premissa visível.</t>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>Depósito: valor_deposito
+Entrega: QT_ENTREGUE · Valor Unitário (contrato)</t>
+        </is>
+      </c>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t>Por mês de tratamento. Depósito mensal = valor_deposito ÷ meses cobertos (6; 3 se oncológico). Compra mensal = (QT_ENTREGUE da última entrega ÷ meses cobertos) × Valor Unitário do contrato. Comparar por princípio ativo. É estimativa: deixar a premissa visível.</t>
         </is>
       </c>
     </row>
@@ -1174,7 +1544,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>Usar a tabela de saídas do SISMAT.</t>
+          <t>Usar a tabela de saídas do SISMAT. O CMM é só de entrega: depósito não tira nada do estoque.</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
@@ -1774,7 +2144,7 @@
     <row r="26">
       <c r="A26" s="9" t="inlineStr">
         <is>
-          <t>Autores (6)</t>
+          <t>Autores – entrega (6a)</t>
         </is>
       </c>
       <c r="B26" s="4" t="n">
@@ -1782,7 +2152,7 @@
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Entrega: na tabela de saídas, programa 486, tipo 6, DT_ENTREGA no período; contar processos distintos por material.</t>
+          <t>Na tabela de saídas, programa 486, tipo 6, DT_ENTREGA no período; contar processos distintos por material.</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
@@ -1799,15 +2169,15 @@
     <row r="27">
       <c r="A27" s="9" t="inlineStr">
         <is>
-          <t>Autores (6)</t>
+          <t>Autores – depósito (6b)</t>
         </is>
       </c>
       <c r="B27" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Depósito: no Fundo, data_pagamento no período e principio_ativo preenchido; contar processos distintos.</t>
+          <t>No Fundo, data_pagamento no período e principio_ativo preenchido; contar processos distintos.</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
@@ -1824,11 +2194,11 @@
     <row r="28">
       <c r="A28" s="9" t="inlineStr">
         <is>
-          <t>Autores (6)</t>
+          <t>Autores – total (6c)</t>
         </is>
       </c>
       <c r="B28" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
@@ -1849,11 +2219,11 @@
     <row r="29">
       <c r="A29" s="9" t="inlineStr">
         <is>
-          <t>Autores (6)</t>
+          <t>Autores – total (6c)</t>
         </is>
       </c>
       <c r="B29" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
@@ -1874,7 +2244,7 @@
     <row r="30">
       <c r="A30" s="9" t="inlineStr">
         <is>
-          <t>Autores (6)</t>
+          <t>Autores – total (6c)</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
@@ -2097,7 +2467,7 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>RedMine</t>
+          <t>RedMine (evitar)</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
@@ -2107,12 +2477,12 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>não usar</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>NUP e nº do processo judicial</t>
+          <t>só o par NUP ↔ nº do processo judicial, e só se não houver outra ponte</t>
         </is>
       </c>
     </row>
@@ -2127,7 +2497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2233,12 +2603,42 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Usar o RedMine para ligar o NUP da triagem ao número do processo judicial.</t>
+          <t>Confirmar se DS_ENTIDADE traz o NUP 00737 (o mesmo da triagem).</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Triagem e Fundo usam números de processo diferentes (4, 5).</t>
+          <t>Se sim, triagem e entrega se ligam direto (4a, 5a, 13b), sem RedMine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Achar uma ponte entre o NUP da triagem e o processo de depósito do Fundo. Última opção: só o par NUP ↔ processo judicial do RedMine.</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>O Fundo não traz o NUP da triagem (4b, 5b).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Advogados com mais processos ficou de fora: o dado só existe no RedMine.</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Evitar o RedMine.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Usa o NUP como chave entre triagem, Fundo e SISMAT no dicionário
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PeYCiidzbNBKwJLDASYnnq
</commit_message>
<xml_diff>
--- a/docs/Dicionario_Painel_Geral_Medicamentos.xlsx
+++ b/docs/Dicionario_Painel_Geral_Medicamentos.xlsx
@@ -622,12 +622,12 @@
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>numero_processo · numero_processo_judicial · data_pagamento · valor_deposito</t>
+          <t>NUP · data_pagamento · valor_deposito</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>Contar processos distintos (numero_processo_judicial) com data_pagamento no período. Valor = soma de valor_deposito.</t>
+          <t>Contar NUPs distintos com data_pagamento no período. Valor = soma de valor_deposito.</t>
         </is>
       </c>
     </row>
@@ -669,7 +669,7 @@
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>Filtrar CO_PROGRAMA_SAUDE = 486 e CO_TIPO_MOVIMENTACAO_ESTOQUE = 6. Contar processos distintos (DS_ENTIDADE) com DT_ENTREGA no período. Quantidade = soma de QT_ENTREGUE; valor = soma de VL_TOTAL_SAIDA.</t>
+          <t>Filtrar CO_PROGRAMA_SAUDE = 486 e CO_TIPO_MOVIMENTACAO_ESTOQUE = 6. Contar NUPs distintos (DS_ENTIDADE) com DT_ENTREGA no período. Quantidade = soma de QT_ENTREGUE; valor = soma de VL_TOTAL_SAIDA.</t>
         </is>
       </c>
     </row>
@@ -713,7 +713,7 @@
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>Ligar NUP da triagem com o processo em DS_ENTIDADE (confirmar se é o NUP 00737). % = NUPs da triagem com entrega ÷ NUPs da triagem.</t>
+          <t>Ligar pelo NUP. % = NUPs da triagem que têm entrega ÷ NUPs da triagem.</t>
         </is>
       </c>
     </row>
@@ -752,12 +752,12 @@
       <c r="G6" s="4" t="inlineStr">
         <is>
           <t>Triagem: NUP
-Fundo: numero_processo · numero_processo_judicial</t>
+Fundo: NUP</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>O Fundo não traz o NUP da triagem (usa o processo de depósito 25000 e o judicial). % = NUPs da triagem com depósito ÷ NUPs da triagem. Para ligar, usar do RedMine apenas o par NUP ↔ nº do processo judicial, se não houver outra ponte.</t>
+          <t>Ligar pelo NUP. % = NUPs da triagem que têm depósito ÷ NUPs da triagem.</t>
         </is>
       </c>
     </row>
@@ -837,7 +837,7 @@
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>DATA (triagem) · DT_ENTREGA · DT_AUTORIZADO</t>
+          <t>NUP · DATA (triagem) · DT_ENTREGA · DT_AUTORIZADO</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
@@ -880,12 +880,12 @@
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>DATA (triagem) · data_pagamento</t>
+          <t>NUP · DATA (triagem) · data_pagamento</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>Entrada → depósito = 1ª data_pagamento do processo − DATA da triagem (depende da ligação de 4b). Mostrar a mediana em dias.</t>
+          <t>Entrada → depósito = 1ª data_pagamento do NUP − DATA da triagem. Mostrar a mediana em dias.</t>
         </is>
       </c>
     </row>
@@ -927,7 +927,7 @@
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>Filtrar 486 e tipo 6, DT_ENTREGA no período. Contar processos distintos (DS_ENTIDADE) por princípio ativo (de-para a partir de CO_MATERIAL).</t>
+          <t>Filtrar 486 e tipo 6, DT_ENTREGA no período. Contar NUPs distintos (DS_ENTIDADE) por princípio ativo (de-para a partir de CO_MATERIAL).</t>
         </is>
       </c>
     </row>
@@ -964,12 +964,12 @@
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>numero_processo_judicial · data_pagamento · principio_ativo</t>
+          <t>NUP · data_pagamento · principio_ativo</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>data_pagamento no período e principio_ativo diferente de "-" e de "NAO SE APLICA". Contar numero_processo_judicial distintos por princípio ativo (de-para).</t>
+          <t>data_pagamento no período e principio_ativo diferente de "-" e de "NAO SE APLICA". Contar NUPs distintos por princípio ativo (de-para).</t>
         </is>
       </c>
     </row>
@@ -1011,7 +1011,7 @@
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>Total = 6a + 6b − autores que aparecem nos dois (mesmo processo nas duas fontes). Pedir ao Vitor a chave que ele já usou.</t>
+          <t>Total = 6a + 6b − NUPs que aparecem nos dois.</t>
         </is>
       </c>
     </row>
@@ -1346,12 +1346,12 @@
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>uf · principio_ativo · numero_processo_judicial</t>
+          <t>uf · principio_ativo · NUP</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>Contar processos distintos por uf e princípio ativo. Por 100 mil hab. = processos da UF ÷ população da UF × 100.000.</t>
+          <t>Contar NUPs distintos por uf e princípio ativo. Por 100 mil hab. = processos da UF ÷ população da UF × 100.000.</t>
         </is>
       </c>
     </row>
@@ -1390,12 +1390,13 @@
       <c r="G21" s="4" t="inlineStr">
         <is>
           <t>Triagem: NUP · UNIDADE FEDERATIVA
-SISMAT: DS_ENTIDADE · CO_MATERIAL</t>
+Fundo: NUP · uf
+SISMAT: DS_ENTIDADE (NUP) · CO_MATERIAL</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>O SISMAT não tem UF. Ligar a saída à triagem pelo NUP e usar UNIDADE FEDERATIVA (preenchida só a partir de abril/2026). Contar processos distintos por UF e princípio ativo.</t>
+          <t>O SISMAT não tem UF. Pegar a UF pelo NUP: na triagem (UNIDADE FEDERATIVA, só a partir de abril/2026) ou no Fundo (uf), quando o mesmo NUP também teve depósito. Contar NUPs distintos por UF e princípio ativo.</t>
         </is>
       </c>
     </row>
@@ -2152,7 +2153,7 @@
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Na tabela de saídas, programa 486, tipo 6, DT_ENTREGA no período; contar processos distintos por material.</t>
+          <t>Na tabela de saídas, programa 486, tipo 6, DT_ENTREGA no período; contar NUPs distintos por material.</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
@@ -2162,7 +2163,7 @@
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>DS_ENTIDADE (processo, confirmar) · DT_ENTREGA · CO_MATERIAL</t>
+          <t>DS_ENTIDADE (NUP) · DT_ENTREGA · CO_MATERIAL</t>
         </is>
       </c>
     </row>
@@ -2177,7 +2178,7 @@
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>No Fundo, data_pagamento no período e principio_ativo preenchido; contar processos distintos.</t>
+          <t>No Fundo, data_pagamento no período e principio_ativo preenchido; contar NUPs distintos.</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
@@ -2187,7 +2188,7 @@
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>numero_processo_judicial · data_pagamento · principio_ativo</t>
+          <t>NUP · data_pagamento · principio_ativo</t>
         </is>
       </c>
     </row>
@@ -2227,7 +2228,7 @@
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Total sem duplicar = entrega + depósito − quem aparece nos dois.</t>
+          <t>Total sem duplicar = entrega + depósito − NUPs que aparecem nos dois.</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
@@ -2237,7 +2238,7 @@
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>mesmo número de processo nas duas fontes</t>
+          <t>NUP</t>
         </is>
       </c>
     </row>
@@ -2279,7 +2280,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -2306,7 +2307,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Identifica o processo por</t>
+          <t>Identifica o processo por (chave: NUP)</t>
         </is>
       </c>
     </row>
@@ -2328,7 +2329,7 @@
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>NUP (00737)</t>
+          <t>NUP</t>
         </is>
       </c>
     </row>
@@ -2350,7 +2351,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>numero_processo_judicial</t>
+          <t>NUP (também traz numero_processo_judicial, usado para o tribunal)</t>
         </is>
       </c>
     </row>
@@ -2372,7 +2373,7 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>DS_ENTIDADE (confirmar)</t>
+          <t>NUP (em DS_ENTIDADE)</t>
         </is>
       </c>
     </row>
@@ -2461,28 +2462,6 @@
       <c r="D8" s="4" t="inlineStr">
         <is>
           <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>RedMine (evitar)</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>baseRedmine</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>não usar</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>só o par NUP ↔ nº do processo judicial, e só se não houver outra ponte</t>
         </is>
       </c>
     </row>
@@ -2497,7 +2476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2548,7 +2527,7 @@
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Confirmar se DS_ENTIDADE traz o processo (2 a 6) e os nomes de saldo e validade (8).</t>
+          <t>Confirmar os nomes de saldo e validade da tabela de estoque (8).</t>
         </is>
       </c>
     </row>
@@ -2603,12 +2582,12 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Confirmar se DS_ENTIDADE traz o NUP 00737 (o mesmo da triagem).</t>
+          <t>Usar o NUP como chave entre triagem, Fundo e SISMAT, no mesmo formato nas três bases (só dígitos).</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Se sim, triagem e entrega se ligam direto (4a, 5a, 13b), sem RedMine.</t>
+          <t>É a ligação do percurso (4, 5), dos autores sem duplicar (6c) e da UF das entregas (13b).</t>
         </is>
       </c>
     </row>
@@ -2618,25 +2597,10 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Achar uma ponte entre o NUP da triagem e o processo de depósito do Fundo. Última opção: só o par NUP ↔ processo judicial do RedMine.</t>
+          <t>Advogados com mais processos ficou de fora: o dado só existe no RedMine.</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>O Fundo não traz o NUP da triagem (4b, 5b).</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>Advogados com mais processos ficou de fora: o dado só existe no RedMine.</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>Evitar o RedMine.</t>
         </is>

</xml_diff>

<commit_message>
Explica cada filtro e cálculo do dicionário em passos
Cada filtro diz a coluna, o valor e o que ele significa; os cálculos viram
passos numerados. A aba de passo a passo vira um glossário dos termos.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PeYCiidzbNBKwJLDASYnnq
</commit_message>
<xml_diff>
--- a/docs/Dicionario_Painel_Geral_Medicamentos.xlsx
+++ b/docs/Dicionario_Painel_Geral_Medicamentos.xlsx
@@ -8,7 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Indicadores" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Passo a passo" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Glossário" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Onde estão os dados" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Antes de começar" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
@@ -496,13 +496,13 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="36" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
-    <col width="42" customWidth="1" min="7" max="7"/>
-    <col width="62" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="90" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -580,12 +580,14 @@
       </c>
       <c r="G2" s="4" t="inlineStr">
         <is>
-          <t>NUP · DATA · GRUPO TEMÁTICO · ORIGEM</t>
+          <t>NUP (número do processo) · DATA (data de entrada) · GRUPO TEMÁTICO</t>
         </is>
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>Contar NUP distintos no período, por mês e por grupo temático.</t>
+          <t>1. Na planilha da triagem, pegar as linhas cuja DATA está dentro do período.
+2. Contar quantos NUPs diferentes existem (o mesmo NUP repetido conta uma vez).
+3. Para os gráficos, fazer a mesma contagem separando por mês da DATA e por GRUPO TEMÁTICO (Geral, Alto Impacto, Oftalmo, Onco).</t>
         </is>
       </c>
     </row>
@@ -602,7 +604,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Cumpridos por depósito</t>
+          <t>Processos cumpridos por depósito</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -612,7 +614,7 @@
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>Quantos foram cumpridos por depósito e quanto custou?</t>
+          <t>Quantos processos receberam depósito e quanto foi depositado?</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
@@ -622,12 +624,14 @@
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>NUP · data_pagamento · valor_deposito</t>
+          <t>NUP · data_pagamento (data do depósito) · valor_deposito (valor em R$)</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>Contar NUPs distintos com data_pagamento no período. Valor = soma de valor_deposito.</t>
+          <t>1. Na planilha do Fundo, pegar as linhas cuja data_pagamento está dentro do período.
+2. Quantidade: contar quantos NUPs diferentes aparecem (um processo com vários depósitos conta uma vez).
+3. Valor: somar a coluna valor_deposito dessas linhas.</t>
         </is>
       </c>
     </row>
@@ -644,7 +648,7 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Cumpridos por entrega</t>
+          <t>Processos cumpridos por entrega</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -654,7 +658,7 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Quantos foram cumpridos com entrega do medicamento e quanto custou?</t>
+          <t>Quantos processos receberam o medicamento e quanto isso custou?</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
@@ -664,12 +668,17 @@
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>DS_ENTIDADE (processo) · DT_ENTREGA · QT_ENTREGUE · VL_TOTAL_SAIDA · CO_PROGRAMA_SAUDE · CO_TIPO_MOVIMENTACAO_ESTOQUE</t>
+          <t>DS_ENTIDADE (traz o NUP) · DT_ENTREGA (data da entrega) · QT_ENTREGUE (quantidade entregue) · VL_TOTAL_SAIDA (valor em R$) · CO_PROGRAMA_SAUDE · CO_TIPO_MOVIMENTACAO_ESTOQUE</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>Filtrar CO_PROGRAMA_SAUDE = 486 e CO_TIPO_MOVIMENTACAO_ESTOQUE = 6. Contar NUPs distintos (DS_ENTIDADE) com DT_ENTREGA no período. Quantidade = soma de QT_ENTREGUE; valor = soma de VL_TOTAL_SAIDA.</t>
+          <t>1. Na tabela de saídas, manter só as linhas em que a coluna CO_PROGRAMA_SAUDE (programa de saúde do SISMAT) é 486, que é o programa "Demanda Judicial – Aquisição" (medicamentos comprados para os processos judiciais). O 546 ("Demanda Judicial – Devolução", material recolhido) fica de fora.
+2. Também manter só as linhas em que a coluna CO_TIPO_MOVIMENTACAO_ESTOQUE (tipo de movimentação do estoque) é 6, que é a saída do medicamento para o autor. Os outros tipos (incineração, troca com a empresa, avaria, doação, transferência para outro programa) ficam de fora. O significado do 6 foi deduzido das observações do SISMAT; confirmar na tabela de domínio.
+3. Manter só as linhas cuja DT_ENTREGA está dentro do período.
+4. Quantidade de processos: contar quantos NUPs diferentes aparecem em DS_ENTIDADE.
+5. Quantidade de medicamento: somar QT_ENTREGUE.
+6. Valor: somar VL_TOTAL_SAIDA.</t>
         </is>
       </c>
     </row>
@@ -686,7 +695,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>% da triagem cumprido por entrega</t>
+          <t>% dos processos da triagem que já receberam entrega</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -696,7 +705,7 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Quanto do que entrou já recebeu o medicamento?</t>
+          <t>Do que entrou, quanto já recebeu o medicamento?</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
@@ -708,12 +717,15 @@
       <c r="G5" s="4" t="inlineStr">
         <is>
           <t>Triagem: NUP
-SISMAT: DS_ENTIDADE</t>
+SISMAT: DS_ENTIDADE (NUP)</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>Ligar pelo NUP. % = NUPs da triagem que têm entrega ÷ NUPs da triagem.</t>
+          <t>1. Pegar a lista de NUPs da triagem no período (indicador 1).
+2. Pegar a lista de NUPs que tiveram entrega (passos 1 a 3 do indicador 3, sem limitar a data da entrega).
+3. Contar quantos NUPs da lista 1 também estão na lista 2.
+4. % = resultado do passo 3 ÷ total de NUPs da lista 1 × 100.</t>
         </is>
       </c>
     </row>
@@ -730,7 +742,7 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>% da triagem cumprido por depósito</t>
+          <t>% dos processos da triagem que já receberam depósito</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -740,7 +752,7 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Quanto do que entrou já recebeu depósito?</t>
+          <t>Do que entrou, quanto já recebeu depósito?</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
@@ -757,7 +769,10 @@
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>Ligar pelo NUP. % = NUPs da triagem que têm depósito ÷ NUPs da triagem.</t>
+          <t>1. Pegar a lista de NUPs da triagem no período (indicador 1).
+2. Pegar a lista de NUPs que aparecem na planilha do Fundo (sem limitar a data do depósito).
+3. Contar quantos NUPs da lista 1 também estão na lista 2.
+4. % = resultado do passo 3 ÷ total de NUPs da lista 1 × 100.</t>
         </is>
       </c>
     </row>
@@ -774,7 +789,7 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>% cumprido no total e processos sem cumprimento</t>
+          <t>% dos processos da triagem já atendidos e lista dos ainda não atendidos</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -784,22 +799,24 @@
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Quanto do que entrou ainda não foi atendido?</t>
+          <t>Do que entrou, quanto já foi atendido de alguma forma e o que falta?</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>Resultado de 4a e 4b</t>
+          <t>Triagem + listas de 4a e 4b</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NUP</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>Cumprido = NUP com entrega OU depósito. Sem cumprimento = NUP sem nenhum dos dois. % = cumpridos ÷ NUPs da triagem.</t>
+          <t>1. Atendido = NUP da triagem que teve entrega OU depósito (está na lista de entrega do 4a, ou na lista de depósito do 4b, ou nas duas).
+2. % atendido = NUPs atendidos ÷ total de NUPs da triagem × 100. Um NUP que teve entrega e depósito conta uma vez só.
+3. Não atendidos = NUPs da triagem que não estão em nenhuma das duas listas. Mostrar a quantidade e a lista.</t>
         </is>
       </c>
     </row>
@@ -816,7 +833,7 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Tempo até a entrega</t>
+          <t>Tempo até a entrega (dias)</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -826,7 +843,7 @@
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Quanto tempo leva para entregar?</t>
+          <t>Quanto tempo leva para o medicamento chegar?</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
@@ -837,12 +854,19 @@
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>NUP · DATA (triagem) · DT_ENTREGA · DT_AUTORIZADO</t>
+          <t>Triagem: NUP · DATA
+SISMAT: DS_ENTIDADE (NUP) · DT_ENTREGA · DT_AUTORIZADO (data em que a saída foi autorizada)</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>Entrada → entrega = 1ª DT_ENTREGA do NUP − DATA da triagem. Autorização → entrega = DT_ENTREGA − DT_AUTORIZADO (descartar datas inválidas como 1-01-01). Mostrar a mediana em dias.</t>
+          <t>Tempo desde a entrada:
+1. Para cada NUP da triagem que teve entrega, pegar a primeira DT_ENTREGA (a mais antiga) desse NUP nas saídas (com os filtros do indicador 3).
+2. Dias = essa DT_ENTREGA − DATA de entrada na triagem.
+3. Mostrar a mediana dos dias (o valor do meio).
+Tempo desde a autorização:
+4. Em cada saída, dias = DT_ENTREGA − DT_AUTORIZADO. Descartar linhas com DT_AUTORIZADO inválida (ex.: 1-01-01).
+5. Mostrar a mediana por medicamento.</t>
         </is>
       </c>
     </row>
@@ -859,7 +883,7 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Tempo até o depósito</t>
+          <t>Tempo até o depósito (dias)</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -869,7 +893,7 @@
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Quanto tempo leva para depositar?</t>
+          <t>Quanto tempo leva para o depósito sair?</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
@@ -880,12 +904,15 @@
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>NUP · DATA (triagem) · data_pagamento</t>
+          <t>Triagem: NUP · DATA
+Fundo: NUP · data_pagamento</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>Entrada → depósito = 1ª data_pagamento do NUP − DATA da triagem. Mostrar a mediana em dias.</t>
+          <t>1. Para cada NUP da triagem que teve depósito, pegar a primeira data_pagamento (a mais antiga) desse NUP no Fundo.
+2. Dias = essa data_pagamento − DATA de entrada na triagem.
+3. Mostrar a mediana dos dias.</t>
         </is>
       </c>
     </row>
@@ -902,7 +929,7 @@
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>Autores atendidos por entrega</t>
+          <t>Autores que receberam o medicamento por entrega</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
@@ -922,12 +949,16 @@
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>DS_ENTIDADE · DT_ENTREGA · CO_MATERIAL</t>
+          <t>DS_ENTIDADE (NUP de cada autor) · DT_ENTREGA · CO_MATERIAL (código do medicamento)</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>Filtrar 486 e tipo 6, DT_ENTREGA no período. Contar NUPs distintos (DS_ENTIDADE) por princípio ativo (de-para a partir de CO_MATERIAL).</t>
+          <t>1. Na tabela de saídas, manter só as linhas em que a coluna CO_PROGRAMA_SAUDE (programa de saúde do SISMAT) é 486, que é o programa "Demanda Judicial – Aquisição" (medicamentos comprados para os processos judiciais). O 546 ("Demanda Judicial – Devolução", material recolhido) fica de fora.
+2. Também manter só as linhas em que a coluna CO_TIPO_MOVIMENTACAO_ESTOQUE (tipo de movimentação do estoque) é 6, que é a saída do medicamento para o autor. Os outros tipos (incineração, troca com a empresa, avaria, doação, transferência para outro programa) ficam de fora. O significado do 6 foi deduzido das observações do SISMAT; confirmar na tabela de domínio.
+3. Manter só as linhas cuja DT_ENTREGA está dentro do período.
+4. Converter CO_MATERIAL em princípio ativo usando a tabela de-para, que converte o código do material do SISMAT (CO_MATERIAL) e o nome escrito no Fundo (principio_ativo) para um mesmo nome padronizado de princípio ativo.
+5. Para cada princípio ativo, contar quantos NUPs diferentes aparecem em DS_ENTIDADE. Cada NUP é um autor.</t>
         </is>
       </c>
     </row>
@@ -944,7 +975,7 @@
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Autores atendidos por depósito</t>
+          <t>Autores que receberam depósito</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
@@ -964,12 +995,15 @@
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>NUP · data_pagamento · principio_ativo</t>
+          <t>NUP (de cada autor) · data_pagamento · principio_ativo</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>data_pagamento no período e principio_ativo diferente de "-" e de "NAO SE APLICA". Contar NUPs distintos por princípio ativo (de-para).</t>
+          <t>1. Na planilha do Fundo, manter só as linhas cuja data_pagamento está dentro do período.
+2. Também manter só as linhas em que a coluna principio_ativo está preenchida (tirar as que têm "-" ou "NAO SE APLICA").
+3. Converter principio_ativo para o nome padronizado usando a tabela de-para, que converte o código do material do SISMAT (CO_MATERIAL) e o nome escrito no Fundo (principio_ativo) para um mesmo nome padronizado de princípio ativo.
+4. Para cada princípio ativo, contar quantos NUPs diferentes aparecem. Cada NUP é um autor.</t>
         </is>
       </c>
     </row>
@@ -986,7 +1020,7 @@
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>Autores atendidos (total sem duplicar)</t>
+          <t>Autores atendidos no total (sem contar ninguém duas vezes)</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
@@ -996,22 +1030,26 @@
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Quantos autores no total, sem contar duas vezes quem recebeu pelas duas vias?</t>
+          <t>Quantos autores no total recebem esse medicamento, por entrega ou por depósito?</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>Resultado de 6a e 6b</t>
+          <t>Listas de 6a e 6b</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NUP · princípio ativo</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>Total = 6a + 6b − NUPs que aparecem nos dois.</t>
+          <t>Um mesmo autor pode ter recebido por entrega e também por depósito; ele deve contar uma vez.
+1. Para cada princípio ativo, juntar a lista de NUPs de entrega (6a) com a lista de NUPs de depósito (6b).
+2. Contar quantos NUPs diferentes existem nessa lista juntada.
+Equivale a: autores por entrega + autores por depósito − autores que aparecem nas duas listas.
+Referência: na primeira versão do Vitor, 3.677 por entrega + 1.843 por depósito − 264 nas duas = 5.256.</t>
         </is>
       </c>
     </row>
@@ -1038,7 +1076,7 @@
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Quanto sai do estoque por mês?</t>
+          <t>Quanto do medicamento sai do estoque por mês?</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
@@ -1048,12 +1086,19 @@
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>QT_ENTREGUE · DT_SAIDA_MATERIAL · CO_MATERIAL · CO_PROGRAMA_SAUDE · CO_TIPO_MOVIMENTACAO_ESTOQUE</t>
+          <t>QT_ENTREGUE · DT_SAIDA_MATERIAL (data da saída do estoque) · CO_MATERIAL · CO_PROGRAMA_SAUDE · CO_TIPO_MOVIMENTACAO_ESTOQUE</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>Soma de QT_ENTREGUE nos últimos 6 meses completos ÷ 6, só 486 e tipo 6. Só entrega: depósito não consome estoque. Ver o passo a passo.</t>
+          <t>Só vale para entrega: depósito não tira nada do estoque.
+1. Na tabela de saídas, manter só as linhas em que a coluna CO_PROGRAMA_SAUDE (programa de saúde do SISMAT) é 486, que é o programa "Demanda Judicial – Aquisição" (medicamentos comprados para os processos judiciais). O 546 ("Demanda Judicial – Devolução", material recolhido) fica de fora.
+2. Também manter só as linhas em que a coluna CO_TIPO_MOVIMENTACAO_ESTOQUE (tipo de movimentação do estoque) é 6, que é a saída do medicamento para o autor. Os outros tipos (incineração, troca com a empresa, avaria, doação, transferência para outro programa) ficam de fora. O significado do 6 foi deduzido das observações do SISMAT; confirmar na tabela de domínio.
+3. Manter só as linhas cuja DT_SAIDA_MATERIAL está nos últimos 6 meses completos (em 19/10/2026: de 01/04/2026 a 30/09/2026; o mês atual fica de fora porque ainda não terminou).
+4. Para cada CO_MATERIAL (cada apresentação do medicamento), somar QT_ENTREGUE.
+5. CMM = essa soma ÷ 6. O resultado é a quantidade que sai por mês, na mesma unidade do estoque.
+Exemplo ilustrativo: 900 unidades em 6 meses → CMM = 150 por mês.
+Opcional: calcular também com 12 meses (soma ÷ 12) para ver se o consumo está subindo ou caindo.</t>
         </is>
       </c>
     </row>
@@ -1070,7 +1115,7 @@
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>Cobertura (meses)</t>
+          <t>Cobertura do estoque (meses)</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
@@ -1086,17 +1131,24 @@
       <c r="F14" s="4" t="inlineStr">
         <is>
           <t>SISMAT · djud.gold.tf_estoque_material_judicial
-+ indicador 7</t>
++ CMM (indicador 7)</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>saldo do lote · validade · CO_PROGRAMA_SAUDE · CO_MATERIAL</t>
+          <t>saldo do lote (quantidade atual) · validade do lote · CO_PROGRAMA_SAUDE · CO_MATERIAL (nomes de saldo e validade a confirmar)</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>Estoque disponível (486, não vencido) ÷ CMM, por apresentação. Ver o passo a passo.</t>
+          <t>1. Na tabela de estoque, manter só as linhas em que a coluna CO_PROGRAMA_SAUDE (programa de saúde do SISMAT) é 486, que é o programa "Demanda Judicial – Aquisição" (medicamentos comprados para os processos judiciais). O 546 ("Demanda Judicial – Devolução", material recolhido) fica de fora.
+2. Manter só os lotes com validade a partir de hoje (lote vencido não pode ser entregue).
+3. Estoque disponível = soma do saldo dos lotes, para cada CO_MATERIAL.
+4. Cobertura = estoque disponível ÷ CMM do mesmo CO_MATERIAL (indicador 7).
+5. Se o CMM for 0, não dividir: mostrar "sem consumo nos últimos 6 meses".
+6. Calcular sempre por apresentação (CO_MATERIAL), porque concentrações diferentes têm unidades diferentes. Na linha do princípio ativo, mostrar a menor cobertura entre as apresentações que tiveram consumo.
+Exemplo ilustrativo: 450 em estoque ÷ CMM 150 = 3 meses.
+Faixas sugeridas: menos de 2 meses = crítica; de 2 a 4 = atenção; 4 ou mais = adequada (validar com a CGLJUD).</t>
         </is>
       </c>
     </row>
@@ -1113,7 +1165,7 @@
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>Ata ou contrato vigente e saldo</t>
+          <t>Ata ou contrato vigente, saldo e vencimento</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
@@ -1123,7 +1175,7 @@
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>Tenho ata vigente? Quanto ainda posso pedir e por quanto tempo isso dura?</t>
+          <t>Tenho ata vigente? Quanto ainda posso pedir à empresa e por quanto tempo isso dura?</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
@@ -1134,13 +1186,20 @@
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>Gerencial: CATMAT · Nº Contrato · Modalidade · Empresa · Status · Data Assinatura · Vigência · Saldo QTD · Saldo (R$) · Valor Unitário
+          <t>Gerencial: CATMAT (código do item) · Nº Contrato · Modalidade · Empresa · Status · Data Assinatura · Vigência (em meses) · Saldo QTD · Saldo (R$) · Valor Unitário
 td_material: CO_CATMAT · CO_MATERIAL</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>Contratos com Status = "Ativo", ligados ao material pelo CATMAT. Saldo em quantidade e em R$, data de fim e saldo em meses (saldo ÷ CMM). Ver o passo a passo.</t>
+          <t>1. Na aba Gerencial da planilha de contratos, manter só as linhas em que a coluna Status é "Ativo" (contrato em vigor).
+2. Ligar cada linha ao medicamento do SISMAT: a coluna CATMAT da planilha corresponde à coluna CO_CATMAT da td_material, que dá o CO_MATERIAL.
+3. Mostrar Nº Contrato, Modalidade, Empresa e Valor Unitário.
+4. Saldo: somar a coluna Saldo QTD (quantidade que ainda pode ser pedida) e a coluna Saldo (R$) dos contratos ativos do mesmo material. Confirmar com a CGLJUD se o saldo certo é Saldo QTD ou Saldo (QTD) Provisório.
+5. Data de fim = Data Assinatura + número de meses da coluna Vigência. Linhas de aditivo (Modalidade "Aditivo Inex", sem vigência) usam a data de fim do contrato original de mesmo Nº Contrato.
+6. Alerta de renovação quando faltar menos de 6 meses para a data de fim (pedido da CGLJUD).
+7. Saldo em meses = Saldo QTD ÷ CMM do mesmo material (indicador 7).
+Conferência (opcional): o número na coluna Empenho da aba Execução aparece na coluna NU_EMPENHO da tabela de entradas do SISMAT (djud.gold.tf_entrada_material_judicial). Ex. real: Vosoritida 0,56 mg, contrato 315/2024, empenho 2024NE000753 – 4.230 unidades entregues na planilha = 4.230 na entrada do SISMAT.</t>
         </is>
       </c>
     </row>
@@ -1157,7 +1216,7 @@
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>Remanejamentos e recolhimentos</t>
+          <t>Remanejamentos e recolhimentos (resumo)</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
@@ -1177,12 +1236,15 @@
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>Situação · Medicamento · Motivo · Local de Coleta</t>
+          <t>Situação (Remanejamento, Recolhimento ou Outro) · Medicamento · Motivo · Local de Coleta</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>Contar registros por Situação (Remanejamento, Recolhimento) e por medicamento no período. Visão resumida; o detalhe fica no painel de remanejamento.</t>
+          <t>1. Na planilha de remanejamento, pegar os registros do período.
+2. Contar os registros com Situação = "Remanejamento" e, à parte, os com Situação = "Recolhimento".
+3. Mostrar a contagem por medicamento (nome padronizado pela de-para) e por Motivo.
+Visão resumida; o detalhe fica no painel de remanejamento que já existe.</t>
         </is>
       </c>
     </row>
@@ -1199,7 +1261,7 @@
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>Incorporado (RENAME)</t>
+          <t>Incorporado ao SUS (RENAME)</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
@@ -1219,12 +1281,13 @@
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>ST_RENAME</t>
+          <t>ST_RENAME (indica se o medicamento está na RENAME, a lista oficial de medicamentos do SUS)</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>Mostrar como coluna e como filtro.</t>
+          <t>1. Para cada CO_MATERIAL, ler a coluna ST_RENAME na td_material.
+2. Mostrar como coluna (Sim/Não) e usar como filtro. Confirmar quais valores a coluna usa (provavelmente S e N).</t>
         </is>
       </c>
     </row>
@@ -1251,7 +1314,7 @@
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>Quanto foi gasto por mês em entregas?</t>
+          <t>Quanto foi gasto por mês entregando medicamento?</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
@@ -1261,12 +1324,14 @@
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>VL_TOTAL_SAIDA · DT_ENTREGA</t>
+          <t>VL_TOTAL_SAIDA (valor em R$) · DT_ENTREGA · CO_PROGRAMA_SAUDE · CO_TIPO_MOVIMENTACAO_ESTOQUE</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>Filtrar 486 e tipo 6. Somar VL_TOTAL_SAIDA por mês de DT_ENTREGA.</t>
+          <t>1. Na tabela de saídas, manter só as linhas em que a coluna CO_PROGRAMA_SAUDE (programa de saúde do SISMAT) é 486, que é o programa "Demanda Judicial – Aquisição" (medicamentos comprados para os processos judiciais). O 546 ("Demanda Judicial – Devolução", material recolhido) fica de fora.
+2. Também manter só as linhas em que a coluna CO_TIPO_MOVIMENTACAO_ESTOQUE (tipo de movimentação do estoque) é 6, que é a saída do medicamento para o autor. Os outros tipos (incineração, troca com a empresa, avaria, doação, transferência para outro programa) ficam de fora. O significado do 6 foi deduzido das observações do SISMAT; confirmar na tabela de domínio.
+3. Para cada mês da DT_ENTREGA, somar VL_TOTAL_SAIDA.</t>
         </is>
       </c>
     </row>
@@ -1293,7 +1358,7 @@
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>Quanto foi gasto por mês em depósitos?</t>
+          <t>Quanto foi gasto por mês com depósitos?</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
@@ -1308,7 +1373,8 @@
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>Somar valor_deposito por mês de data_pagamento. Mostrar ao lado de 12a.</t>
+          <t>1. Na planilha do Fundo, para cada mês da data_pagamento, somar valor_deposito.
+2. Mostrar no mesmo gráfico do 12a, lado a lado.</t>
         </is>
       </c>
     </row>
@@ -1335,23 +1401,25 @@
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>Quais medicamentos mais judicializados em cada UF? E por 100 mil habitantes?</t>
+          <t>Quais medicamentos têm mais processos em cada UF? E por 100 mil habitantes?</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
           <t>Fundo · planilha depositos_tratados
-+ população do IBGE</t>
++ população por UF do IBGE</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>uf · principio_ativo · NUP</t>
+          <t>uf (estado do depósito) · principio_ativo · NUP</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>Contar NUPs distintos por uf e princípio ativo. Por 100 mil hab. = processos da UF ÷ população da UF × 100.000.</t>
+          <t>1. Na planilha do Fundo, manter as linhas do período e manter só as linhas em que a coluna principio_ativo está preenchida (tirar as que têm "-" ou "NAO SE APLICA").
+2. Para cada uf e princípio ativo (padronizado), contar quantos NUPs diferentes aparecem.
+3. Por 100 mil habitantes = NUPs da UF ÷ população da UF (IBGE) × 100.000.</t>
         </is>
       </c>
     </row>
@@ -1384,6 +1452,7 @@
       <c r="F21" s="4" t="inlineStr">
         <is>
           <t>Planilha da Triagem (CGAJUD)
+Fundo · planilha depositos_tratados
 SISMAT · djud.gold.tf_saida_material_judicial</t>
         </is>
       </c>
@@ -1396,7 +1465,10 @@
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>O SISMAT não tem UF. Pegar a UF pelo NUP: na triagem (UNIDADE FEDERATIVA, só a partir de abril/2026) ou no Fundo (uf), quando o mesmo NUP também teve depósito. Contar NUPs distintos por UF e princípio ativo.</t>
+          <t>O SISMAT não tem o estado do autor.
+1. Pegar as entregas com os filtros do indicador 3.
+2. Para cada NUP, buscar o estado: primeiro na coluna UNIDADE FEDERATIVA da triagem (preenchida só a partir de abril/2026); se não tiver, na coluna uf do Fundo, quando o mesmo NUP também teve depósito.
+3. Para cada estado e princípio ativo, contar quantos NUPs diferentes aparecem. NUP sem estado encontrado vai para "UF não identificada".</t>
         </is>
       </c>
     </row>
@@ -1423,7 +1495,7 @@
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>Quais tribunais concentram mais ações e valor?</t>
+          <t>Quais tribunais concentram mais processos e mais valor?</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
@@ -1433,12 +1505,14 @@
       </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
-          <t>numero_processo_judicial · valor_deposito</t>
+          <t>numero_processo_judicial (número do processo na Justiça, 20 dígitos) · valor_deposito</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>Tribunal = dígitos 14 a 16 do número do processo judicial (J + TR). Contar processos e somar valor_deposito por tribunal. Só depósito: o SISMAT não traz o número judicial.</t>
+          <t>1. Na planilha do Fundo, pegar os dígitos 14 a 16 de numero_processo_judicial: o 14º é o ramo da Justiça (4 = Federal, 8 = Estadual) e o 15º e 16º são o tribunal ou região (ex.: 4 + 01 = TRF da 1ª Região).
+2. Para cada tribunal, contar NUPs diferentes e somar valor_deposito.
+Só para depósito: o SISMAT não traz o número do processo na Justiça.</t>
         </is>
       </c>
     </row>
@@ -1455,7 +1529,7 @@
       </c>
       <c r="C23" s="8" t="inlineStr">
         <is>
-          <t>Depositar ou comprar</t>
+          <t>Depositar ou comprar: qual sai mais caro</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
@@ -1465,24 +1539,30 @@
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>Para o mesmo medicamento, sai mais caro depositar ou comprar?</t>
+          <t>Para o mesmo medicamento, sai mais caro depositar ou comprar e entregar?</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
           <t>Fundo · planilha depositos_tratados
+SISMAT · djud.gold.tf_saida_material_judicial
 Planilha Gestão de Contratos (SharePoint da CGLJUD) · abas Gerencial e Execução</t>
         </is>
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
-          <t>Depósito: valor_deposito
-Entrega: QT_ENTREGUE · Valor Unitário (contrato)</t>
+          <t>Fundo: valor_deposito · NUP
+SISMAT: QT_ENTREGUE · DS_ENTIDADE (NUP)
+Contratos: Valor Unitário</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>Por mês de tratamento. Depósito mensal = valor_deposito ÷ meses cobertos (6; 3 se oncológico). Compra mensal = (QT_ENTREGUE da última entrega ÷ meses cobertos) × Valor Unitário do contrato. Comparar por princípio ativo. É estimativa: deixar a premissa visível.</t>
+          <t>O Fundo não informa a quantidade de medicamento de cada depósito, então a comparação é por mês de tratamento.
+1. Depósito por mês: valor_deposito ÷ meses que ele cobre (6 meses; 3 para oncológicos).
+2. Compra por mês: pegar a última entrega de cada autor (QT_ENTREGUE), dividir pelos meses que ela cobre (6 ou 3) e multiplicar pelo Valor Unitário do contrato vigente.
+3. Comparar a média do passo 1 com a média do passo 2, por princípio ativo.
+É uma estimativa: mostrar no painel a premissa de 6 e 3 meses.</t>
         </is>
       </c>
     </row>
@@ -1497,775 +1577,166 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="70" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="48" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="110" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Indicador</t>
+          <t>Termo</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Passo</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>O que fazer</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Tabela</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Campos</t>
+          <t>O que significa</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="9" t="inlineStr">
         <is>
-          <t>CMM (7)</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>Usar a tabela de saídas do SISMAT. O CMM é só de entrega: depósito não tira nada do estoque.</t>
-        </is>
-      </c>
-      <c r="D2" s="4" t="inlineStr">
-        <is>
-          <t>djud.gold.tf_saida_material_judicial</t>
-        </is>
-      </c>
-      <c r="E2" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
+          <t>NUP</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>Número do processo no SEI. É a chave que liga a triagem, o Fundo e o SISMAT.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
         <is>
-          <t>CMM (7)</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>Manter só o programa de aquisição judicial.</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>idem</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>CO_PROGRAMA_SAUDE = 486</t>
+          <t>CO_PROGRAMA_SAUDE</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Coluna do SISMAT com o programa de saúde a que o medicamento pertence. 486 = "Demanda Judicial – Aquisição" (comprado para processos judiciais; é o que interessa). 546 = "Demanda Judicial – Devolução" (recolhido, não reutilizável).</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="9" t="inlineStr">
         <is>
-          <t>CMM (7)</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>Manter só dispensação para autor (tira incineração, troca, avaria, doação, transferência).</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>idem</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>CO_TIPO_MOVIMENTACAO_ESTOQUE = 6 (confirmar na tabela de domínio)</t>
+          <t>CO_TIPO_MOVIMENTACAO_ESTOQUE</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Coluna do SISMAT com o tipo de movimentação. Nas saídas, 6 = saída do medicamento para o autor (a que conta como entrega e consumo). Outros valores vistos: 43 e 25 incineração, 34 troca com a empresa, 28 avaria, 7 amostras para análise, 26 doação, 39 transferência para outro programa. Significados deduzidos das observações; confirmar.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
         <is>
-          <t>CMM (7)</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>Pegar os últimos 6 meses completos. Ex.: em 19/10/2026 → de 01/04/2026 a 30/09/2026.</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>idem</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>DT_SAIDA_MATERIAL</t>
+          <t>CO_MATERIAL</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Código do medicamento no SISMAT. Cada concentração ou forma é um código diferente (ex.: Vosoritida 0,4 mg e 0,56 mg).</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="9" t="inlineStr">
         <is>
-          <t>CMM (7)</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>Somar a quantidade por material.</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>idem</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>SOMA(QT_ENTREGUE) por CO_MATERIAL</t>
+          <t>Apresentação</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Uma concentração/forma específica do medicamento (um CO_MATERIAL).</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
         <is>
-          <t>CMM (7)</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>Dividir por 6. Resultado = unidades por mês, na mesma unidade do estoque.</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>CMM = soma ÷ 6</t>
+          <t>Princípio ativo</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>A substância do medicamento, juntando todas as apresentações (ex.: VOSORITIDA).</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
         <is>
-          <t>CMM (7)</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>Opcional: calcular também com 12 meses (÷ 12) para ver se o consumo está subindo ou caindo.</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
+          <t>Tabela de-para</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Tabela a criar que converte o CO_MATERIAL do SISMAT e o nome escrito no Fundo e no remanejamento para um mesmo nome padronizado de princípio ativo.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
         <is>
-          <t>CMM (7)</t>
+          <t>CATMAT</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Exemplo</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>Ilustrativo: 900 unidades saíram entre abril e setembro → CMM = 900 ÷ 6 = 150 por mês.</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
+          <t>Código do item no catálogo de materiais do governo. Liga a planilha de contratos (coluna CATMAT) ao SISMAT (coluna CO_CATMAT).</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
         <is>
-          <t>Cobertura (8)</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>Estoque disponível: somar o saldo dos lotes do programa 486 com validade a partir de hoje.</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>djud.gold.tf_estoque_material_judicial</t>
-        </is>
-      </c>
-      <c r="E10" s="4" t="inlineStr">
-        <is>
-          <t>saldo do lote · validade · CO_PROGRAMA_SAUDE · CO_MATERIAL (nomes de saldo e validade a confirmar com DESCRIBE)</t>
+          <t>CMM</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Consumo médio mensal: quanto do medicamento sai do estoque por mês, em média.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
         <is>
-          <t>Cobertura (8)</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>Dividir pelo CMM do mesmo material.</t>
-        </is>
-      </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>Cobertura = estoque disponível ÷ CMM</t>
+          <t>Cobertura</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Quantos meses o estoque atual dura no ritmo do CMM.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
         <is>
-          <t>Cobertura (8)</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>Se o CMM for 0, não dividir: mostrar "sem consumo nos últimos 6 meses".</t>
-        </is>
-      </c>
-      <c r="D12" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E12" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
+          <t>Mediana</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>O valor do meio quando os tempos são colocados em ordem. Menos afetada por casos extremos do que a média.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="9" t="inlineStr">
         <is>
-          <t>Cobertura (8)</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>Calcular por apresentação (CO_MATERIAL), porque concentrações diferentes têm unidades diferentes. Na linha do princípio ativo, mostrar a menor cobertura entre as apresentações que tiveram consumo.</t>
-        </is>
-      </c>
-      <c r="D13" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E13" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="9" t="inlineStr">
-        <is>
-          <t>Cobertura (8)</t>
-        </is>
-      </c>
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>Exemplo</t>
-        </is>
-      </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t>Ilustrativo: 450 em estoque ÷ CMM 150 = 3 meses.</t>
-        </is>
-      </c>
-      <c r="D14" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="9" t="inlineStr">
-        <is>
-          <t>Cobertura (8)</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>Faixas</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>Crítica: menos de 2 meses · Atenção: 2 a 4 · Adequada: 4 ou mais (validar com a CGLJUD).</t>
-        </is>
-      </c>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E15" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="9" t="inlineStr">
-        <is>
-          <t>Atas (9)</t>
-        </is>
-      </c>
-      <c r="B16" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>Fonte: planilha Gestão de Contratos, mantida à mão pela equipe de gestão contratual da CGLJUD no SharePoint. Enquanto o acesso automático ao SharePoint não sai, usar a cópia recebida.</t>
-        </is>
-      </c>
-      <c r="D16" s="4" t="inlineStr">
-        <is>
-          <t>Gestão de Contratos · aba Gerencial (uma linha por contrato × item)</t>
-        </is>
-      </c>
-      <c r="E16" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="9" t="inlineStr">
-        <is>
-          <t>Atas (9)</t>
-        </is>
-      </c>
-      <c r="B17" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>Manter só contratos vigentes.</t>
-        </is>
-      </c>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
-          <t>aba Gerencial</t>
-        </is>
-      </c>
-      <c r="E17" s="4" t="inlineStr">
-        <is>
-          <t>Status = "Ativo"</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="9" t="inlineStr">
-        <is>
-          <t>Atas (9)</t>
-        </is>
-      </c>
-      <c r="B18" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="C18" s="4" t="inlineStr">
-        <is>
-          <t>Ligar ao material do SISMAT pelo CATMAT (padronizar: só dígitos, sem zeros à esquerda).</t>
-        </is>
-      </c>
-      <c r="D18" s="4" t="inlineStr">
-        <is>
-          <t>aba Gerencial + dbsismat.bronze.td_material</t>
-        </is>
-      </c>
-      <c r="E18" s="4" t="inlineStr">
-        <is>
-          <t>CATMAT = td_material.CO_CATMAT → CO_MATERIAL</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="9" t="inlineStr">
-        <is>
-          <t>Atas (9)</t>
-        </is>
-      </c>
-      <c r="B19" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="C19" s="4" t="inlineStr">
-        <is>
-          <t>Mostrar o contrato: número, modalidade, empresa e preço.</t>
-        </is>
-      </c>
-      <c r="D19" s="4" t="inlineStr">
-        <is>
-          <t>aba Gerencial</t>
-        </is>
-      </c>
-      <c r="E19" s="4" t="inlineStr">
-        <is>
-          <t>Nº Contrato · Modalidade · Empresa · Valor Unitário</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="9" t="inlineStr">
-        <is>
-          <t>Atas (9)</t>
-        </is>
-      </c>
-      <c r="B20" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="C20" s="4" t="inlineStr">
-        <is>
-          <t>Saldo: somar o saldo dos contratos ativos do material.</t>
-        </is>
-      </c>
-      <c r="D20" s="4" t="inlineStr">
-        <is>
-          <t>aba Gerencial</t>
-        </is>
-      </c>
-      <c r="E20" s="4" t="inlineStr">
-        <is>
-          <t>Saldo QTD (ou Saldo (QTD) Provisório: confirmar qual) · Saldo (R$)</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="9" t="inlineStr">
-        <is>
-          <t>Atas (9)</t>
-        </is>
-      </c>
-      <c r="B21" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="C21" s="4" t="inlineStr">
-        <is>
-          <t>Data de fim = data de assinatura + vigência em meses. Aditivos (Modalidade "Aditivo Inex", sem vigência) usam a data de fim do contrato original de mesmo Nº Contrato.</t>
-        </is>
-      </c>
-      <c r="D21" s="4" t="inlineStr">
-        <is>
-          <t>aba Gerencial</t>
-        </is>
-      </c>
-      <c r="E21" s="4" t="inlineStr">
-        <is>
-          <t>Data Assinatura · Vigência · Nº Contrato · Modalidade</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="9" t="inlineStr">
-        <is>
-          <t>Atas (9)</t>
-        </is>
-      </c>
-      <c r="B22" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="C22" s="4" t="inlineStr">
-        <is>
-          <t>Alerta de renovação: data de fim em menos de 6 meses (pedido da CGLJUD).</t>
-        </is>
-      </c>
-      <c r="D22" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E22" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="9" t="inlineStr">
-        <is>
-          <t>Atas (9)</t>
-        </is>
-      </c>
-      <c r="B23" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="C23" s="4" t="inlineStr">
-        <is>
-          <t>Saldo em meses = saldo em quantidade ÷ CMM do material.</t>
-        </is>
-      </c>
-      <c r="D23" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E23" s="4" t="inlineStr">
-        <is>
-          <t>Saldo QTD ÷ CMM</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="9" t="inlineStr">
-        <is>
-          <t>Atas (9)</t>
-        </is>
-      </c>
-      <c r="B24" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="C24" s="4" t="inlineStr">
-        <is>
-          <t>Conferência: o empenho da aba Execução deve bater com a entrada no SISMAT.</t>
-        </is>
-      </c>
-      <c r="D24" s="4" t="inlineStr">
-        <is>
-          <t>aba Execução + djud.gold.tf_entrada_material_judicial</t>
-        </is>
-      </c>
-      <c r="E24" s="4" t="inlineStr">
-        <is>
-          <t>Empenho = NU_EMPENHO · Quantidade Entregue ≈ QT_ENTRADA</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="9" t="inlineStr">
-        <is>
-          <t>Atas (9)</t>
-        </is>
-      </c>
-      <c r="B25" s="4" t="inlineStr">
-        <is>
-          <t>Exemplo</t>
-        </is>
-      </c>
-      <c r="C25" s="4" t="inlineStr">
-        <is>
-          <t>Real: Vosoritida 0,56 mg, contrato 315/2024, empenho 2024NE000753 – 4.230 entregues na planilha = 4.230 na entrada do SISMAT.</t>
-        </is>
-      </c>
-      <c r="D25" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E25" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="9" t="inlineStr">
-        <is>
-          <t>Autores – entrega (6a)</t>
-        </is>
-      </c>
-      <c r="B26" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="C26" s="4" t="inlineStr">
-        <is>
-          <t>Na tabela de saídas, programa 486, tipo 6, DT_ENTREGA no período; contar NUPs distintos por material.</t>
-        </is>
-      </c>
-      <c r="D26" s="4" t="inlineStr">
-        <is>
-          <t>djud.gold.tf_saida_material_judicial</t>
-        </is>
-      </c>
-      <c r="E26" s="4" t="inlineStr">
-        <is>
-          <t>DS_ENTIDADE (NUP) · DT_ENTREGA · CO_MATERIAL</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="9" t="inlineStr">
-        <is>
-          <t>Autores – depósito (6b)</t>
-        </is>
-      </c>
-      <c r="B27" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="C27" s="4" t="inlineStr">
-        <is>
-          <t>No Fundo, data_pagamento no período e principio_ativo preenchido; contar NUPs distintos.</t>
-        </is>
-      </c>
-      <c r="D27" s="4" t="inlineStr">
-        <is>
-          <t>depositos_tratados</t>
-        </is>
-      </c>
-      <c r="E27" s="4" t="inlineStr">
-        <is>
-          <t>NUP · data_pagamento · principio_ativo</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="9" t="inlineStr">
-        <is>
-          <t>Autores – total (6c)</t>
-        </is>
-      </c>
-      <c r="B28" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="C28" s="4" t="inlineStr">
-        <is>
-          <t>Levar os dois para o mesmo princípio ativo pela tabela de-para.</t>
-        </is>
-      </c>
-      <c r="D28" s="4" t="inlineStr">
-        <is>
-          <t>de-para (a criar)</t>
-        </is>
-      </c>
-      <c r="E28" s="4" t="inlineStr">
-        <is>
-          <t>CO_MATERIAL → princípio ativo; principio_ativo do Fundo → princípio ativo</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="9" t="inlineStr">
-        <is>
-          <t>Autores – total (6c)</t>
-        </is>
-      </c>
-      <c r="B29" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="C29" s="4" t="inlineStr">
-        <is>
-          <t>Total sem duplicar = entrega + depósito − NUPs que aparecem nos dois.</t>
-        </is>
-      </c>
-      <c r="D29" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E29" s="4" t="inlineStr">
-        <is>
-          <t>NUP</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="9" t="inlineStr">
-        <is>
-          <t>Autores – total (6c)</t>
-        </is>
-      </c>
-      <c r="B30" s="4" t="inlineStr">
-        <is>
-          <t>Referência</t>
-        </is>
-      </c>
-      <c r="C30" s="4" t="inlineStr">
-        <is>
-          <t>Na primeira versão do Vitor: 3.677 por entrega + 1.843 por depósito − 264 nos dois = 5.256. Pedir a ele a chave usada.</t>
-        </is>
-      </c>
-      <c r="D30" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E30" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
+          <t>Período</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>O intervalo de datas escolhido no filtro do painel.</t>
         </is>
       </c>
     </row>
@@ -2537,12 +2008,12 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Confirmar o significado de CO_TIPO_MOVIMENTACAO_ESTOQUE = 6.</t>
+          <t>Confirmar, na tabela de domínio do SISMAT, que o valor 6 da coluna CO_TIPO_MOVIMENTACAO_ESTOQUE é a saída para o autor.</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>É o filtro que separa consumo de perdas e trocas (3, 7).</t>
+          <t>É o filtro que separa entrega e consumo de incineração, troca e avaria (indicadores 3, 6a, 7, 12a).</t>
         </is>
       </c>
     </row>

</xml_diff>